<commit_message>
update to plots and stilabilty deriv
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -419,10 +419,10 @@
     <t>Wing area</t>
   </si>
   <si>
-    <t>CM_0</t>
-  </si>
-  <si>
-    <t>Moment Coefficient</t>
+    <t>CM_ac_w</t>
+  </si>
+  <si>
+    <t>Moment Coefficient at AC, wing</t>
   </si>
   <si>
     <t>XFLR5</t>

</xml_diff>

<commit_message>
pushing a5b mir will never see this lol
thanks
</commit_message>
<xml_diff>
--- a/SizingParams.xlsx
+++ b/SizingParams.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hudson/Documents/GitHub/451-DBF-Team01/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ceaa8977d2236823/Documents/GitHub/451-DBF-Team01/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB30DBF-D90C-D04A-9CE1-D2D257DE167B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{8DB30DBF-D90C-D04A-9CE1-D2D257DE167B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08EDA64E-72B2-45A2-9A9B-BAEF15EC70EF}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INPUTS" sheetId="1" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="160">
   <si>
     <t>Parameter</t>
   </si>
@@ -514,6 +514,27 @@
   </si>
   <si>
     <t>CM_ac_w</t>
+  </si>
+  <si>
+    <t>SM</t>
+  </si>
+  <si>
+    <t>--</t>
+  </si>
+  <si>
+    <t>Static Margin</t>
+  </si>
+  <si>
+    <t>Wingspan</t>
+  </si>
+  <si>
+    <t>Wing Span</t>
+  </si>
+  <si>
+    <t>Fuselage Thickness</t>
+  </si>
+  <si>
+    <t>t_fuselage</t>
   </si>
 </sst>
 </file>
@@ -695,7 +716,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
@@ -718,6 +739,7 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,16 +878,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>540205</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>131987</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>9151</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>141220</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>314597</xdr:colOff>
-      <xdr:row>54</xdr:row>
-      <xdr:rowOff>99030</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>43963</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>67330</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -888,8 +910,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7449005" y="7472587"/>
-          <a:ext cx="4486093" cy="2536254"/>
+          <a:off x="8017478" y="6918624"/>
+          <a:ext cx="3639658" cy="2307360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2393,17 +2415,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Q129"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.55" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="25.83203125" style="1" customWidth="1"/>
-    <col min="6" max="18" width="8.83203125" style="1" customWidth="1"/>
-    <col min="19" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="11.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="1" customWidth="1"/>
+    <col min="4" max="5" width="25.77734375" style="1" customWidth="1"/>
+    <col min="6" max="18" width="8.77734375" style="1" customWidth="1"/>
+    <col min="19" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2434,7 +2456,7 @@
       <c r="P1" s="4"/>
       <c r="Q1" s="4"/>
     </row>
-    <row r="2" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>6</v>
       </c>
@@ -2465,7 +2487,7 @@
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
     </row>
-    <row r="3" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>11</v>
       </c>
@@ -2494,7 +2516,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
@@ -2523,7 +2545,7 @@
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
     </row>
-    <row r="5" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
@@ -2554,7 +2576,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -2585,7 +2607,7 @@
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
     </row>
-    <row r="7" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>26</v>
       </c>
@@ -2614,12 +2636,13 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="B8" s="9">
-        <v>5</v>
+        <f>B51/B42</f>
+        <v>4.7168676768718001</v>
       </c>
       <c r="C8" s="7" t="s">
         <v>19</v>
@@ -2645,13 +2668,13 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
-    <row r="9" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>33</v>
       </c>
       <c r="B9" s="10" cm="1">
         <f t="array" ref="B9">1/(PI()*B7*B8)</f>
-        <v>9.0945681766797334E-2</v>
+        <v>9.6404741448155279E-2</v>
       </c>
       <c r="C9" s="7" t="s">
         <v>19</v>
@@ -2675,7 +2698,7 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
     </row>
-    <row r="10" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>36</v>
       </c>
@@ -2704,7 +2727,7 @@
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
     </row>
-    <row r="11" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>39</v>
       </c>
@@ -2735,7 +2758,7 @@
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
     </row>
-    <row r="12" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>43</v>
       </c>
@@ -2767,7 +2790,7 @@
       <c r="P12" s="4"/>
       <c r="Q12" s="4"/>
     </row>
-    <row r="13" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>47</v>
       </c>
@@ -2799,7 +2822,7 @@
       <c r="P13" s="4"/>
       <c r="Q13" s="4"/>
     </row>
-    <row r="14" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>51</v>
       </c>
@@ -2830,13 +2853,13 @@
       <c r="P14" s="4"/>
       <c r="Q14" s="4"/>
     </row>
-    <row r="15" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="21" t="s">
         <v>151</v>
       </c>
       <c r="B15" s="10" cm="1">
         <f t="array" ref="B15">B14+B9*B10^2</f>
-        <v>4.8185111359011761E-2</v>
+        <v>4.8676426730333976E-2</v>
       </c>
       <c r="C15" s="7" t="s">
         <v>19</v>
@@ -2860,13 +2883,13 @@
       <c r="P15" s="4"/>
       <c r="Q15" s="4"/>
     </row>
-    <row r="16" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>57</v>
       </c>
       <c r="B16" s="10" cm="1">
         <f t="array" ref="B16">B14+B9*B12^2</f>
-        <v>4.8185111359011761E-2</v>
+        <v>4.8676426730333976E-2</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>19</v>
@@ -2892,13 +2915,13 @@
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
     </row>
-    <row r="17" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>60</v>
       </c>
       <c r="B17" s="10" cm="1">
         <f t="array" ref="B17">B16-B5*B12</f>
-        <v>3.3185111359011761E-2</v>
+        <v>3.3676426730333976E-2</v>
       </c>
       <c r="C17" s="7" t="s">
         <v>19</v>
@@ -2922,13 +2945,13 @@
       <c r="P17" s="4"/>
       <c r="Q17" s="4"/>
     </row>
-    <row r="18" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>63</v>
       </c>
       <c r="B18" s="12" cm="1">
         <f t="array" ref="B18">B10/B15</f>
-        <v>6.2259895544247374</v>
+        <v>6.1631475470044563</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>19</v>
@@ -2952,7 +2975,7 @@
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
     </row>
-    <row r="19" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>66</v>
       </c>
@@ -2981,7 +3004,7 @@
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
     </row>
-    <row r="20" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>69</v>
       </c>
@@ -3010,7 +3033,7 @@
       <c r="P20" s="4"/>
       <c r="Q20" s="4"/>
     </row>
-    <row r="21" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
         <v>71</v>
       </c>
@@ -3040,7 +3063,7 @@
       <c r="P21" s="4"/>
       <c r="Q21" s="4"/>
     </row>
-    <row r="22" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>73</v>
       </c>
@@ -3070,7 +3093,7 @@
       <c r="P22" s="4"/>
       <c r="Q22" s="4"/>
     </row>
-    <row r="23" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>76</v>
       </c>
@@ -3098,7 +3121,7 @@
       <c r="P23" s="4"/>
       <c r="Q23" s="4"/>
     </row>
-    <row r="24" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>78</v>
       </c>
@@ -3128,7 +3151,7 @@
       <c r="P24" s="4"/>
       <c r="Q24" s="4"/>
     </row>
-    <row r="25" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>81</v>
       </c>
@@ -3157,7 +3180,7 @@
       <c r="P25" s="4"/>
       <c r="Q25" s="4"/>
     </row>
-    <row r="26" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>84</v>
       </c>
@@ -3186,7 +3209,7 @@
       <c r="P26" s="4"/>
       <c r="Q26" s="4"/>
     </row>
-    <row r="27" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>87</v>
       </c>
@@ -3214,7 +3237,7 @@
       <c r="P27" s="4"/>
       <c r="Q27" s="4"/>
     </row>
-    <row r="28" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>90</v>
       </c>
@@ -3243,7 +3266,7 @@
       <c r="P28" s="4"/>
       <c r="Q28" s="4"/>
     </row>
-    <row r="29" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>93</v>
       </c>
@@ -3272,7 +3295,7 @@
       <c r="P29" s="4"/>
       <c r="Q29" s="4"/>
     </row>
-    <row r="30" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
         <v>96</v>
       </c>
@@ -3301,7 +3324,7 @@
       <c r="P30" s="4"/>
       <c r="Q30" s="4"/>
     </row>
-    <row r="31" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>98</v>
       </c>
@@ -3330,7 +3353,7 @@
       <c r="P31" s="4"/>
       <c r="Q31" s="4"/>
     </row>
-    <row r="32" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>101</v>
       </c>
@@ -3359,7 +3382,7 @@
       <c r="P32" s="4"/>
       <c r="Q32" s="4"/>
     </row>
-    <row r="33" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
         <v>104</v>
       </c>
@@ -3387,7 +3410,7 @@
       <c r="P33" s="4"/>
       <c r="Q33" s="4"/>
     </row>
-    <row r="34" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
         <v>106</v>
       </c>
@@ -3416,12 +3439,12 @@
       <c r="P34" s="4"/>
       <c r="Q34" s="4"/>
     </row>
-    <row r="35" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
         <v>109</v>
       </c>
       <c r="B35" s="6">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C35" s="7" t="s">
         <v>110</v>
@@ -3443,7 +3466,7 @@
       <c r="P35" s="4"/>
       <c r="Q35" s="4"/>
     </row>
-    <row r="36" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
         <v>112</v>
       </c>
@@ -3470,7 +3493,7 @@
       <c r="P36" s="4"/>
       <c r="Q36" s="4"/>
     </row>
-    <row r="37" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>115</v>
       </c>
@@ -3497,7 +3520,7 @@
       <c r="P37" s="4"/>
       <c r="Q37" s="4"/>
     </row>
-    <row r="38" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
         <v>117</v>
       </c>
@@ -3526,7 +3549,7 @@
       <c r="P38" s="4"/>
       <c r="Q38" s="4"/>
     </row>
-    <row r="39" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
         <v>121</v>
       </c>
@@ -3554,13 +3577,13 @@
       <c r="P39" s="4"/>
       <c r="Q39" s="4"/>
     </row>
-    <row r="40" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="B40" s="17" cm="1">
-        <f t="array" ref="B40">B39/B35</f>
-        <v>0.43654500000000007</v>
+      <c r="B40" s="17">
+        <f>B39/B35</f>
+        <v>0.459521052631579</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>125</v>
@@ -3582,7 +3605,7 @@
       <c r="P40" s="4"/>
       <c r="Q40" s="4"/>
     </row>
-    <row r="41" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
         <v>152</v>
       </c>
@@ -3611,12 +3634,13 @@
       <c r="P41" s="4"/>
       <c r="Q41" s="4"/>
     </row>
-    <row r="42" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>129</v>
       </c>
       <c r="B42" s="18">
-        <v>0.29099999999999998</v>
+        <f>B40/(B51-B52)</f>
+        <v>0.31800764887998545</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="2" t="s">
@@ -3636,7 +3660,7 @@
       <c r="P42" s="4"/>
       <c r="Q42" s="4"/>
     </row>
-    <row r="43" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>131</v>
       </c>
@@ -3663,7 +3687,7 @@
       <c r="P43" s="4"/>
       <c r="Q43" s="4"/>
     </row>
-    <row r="44" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="19" t="s">
         <v>134</v>
       </c>
@@ -3690,12 +3714,12 @@
       <c r="P44" s="4"/>
       <c r="Q44" s="4"/>
     </row>
-    <row r="45" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>137</v>
       </c>
       <c r="B45" s="18">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>19</v>
@@ -3719,7 +3743,7 @@
       <c r="P45" s="4"/>
       <c r="Q45" s="4"/>
     </row>
-    <row r="46" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>140</v>
       </c>
@@ -3748,7 +3772,7 @@
       <c r="P46" s="4"/>
       <c r="Q46" s="4"/>
     </row>
-    <row r="47" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>142</v>
       </c>
@@ -3777,7 +3801,7 @@
       <c r="P47" s="4"/>
       <c r="Q47" s="4"/>
     </row>
-    <row r="48" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>145</v>
       </c>
@@ -3806,7 +3830,7 @@
       <c r="P48" s="4"/>
       <c r="Q48" s="4"/>
     </row>
-    <row r="49" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="20" t="s">
         <v>148</v>
       </c>
@@ -3835,11 +3859,19 @@
       <c r="P49" s="4"/>
       <c r="Q49" s="4"/>
     </row>
-    <row r="50" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
+    <row r="50" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B50" s="4">
+        <v>0.15</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
       <c r="G50" s="4"/>
@@ -3854,11 +3886,19 @@
       <c r="P50" s="4"/>
       <c r="Q50" s="4"/>
     </row>
-    <row r="51" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="4"/>
-      <c r="B51" s="4"/>
-      <c r="C51" s="4"/>
-      <c r="D51" s="4"/>
+    <row r="51" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B51" s="4">
+        <v>1.5</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>157</v>
+      </c>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
       <c r="G51" s="4"/>
@@ -3873,11 +3913,19 @@
       <c r="P51" s="4"/>
       <c r="Q51" s="4"/>
     </row>
-    <row r="52" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="4"/>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
+    <row r="52" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="B52" s="4">
+        <v>5.5E-2</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>158</v>
+      </c>
       <c r="E52" s="4"/>
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
@@ -3892,7 +3940,7 @@
       <c r="P52" s="4"/>
       <c r="Q52" s="4"/>
     </row>
-    <row r="53" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3911,7 +3959,7 @@
       <c r="P53" s="4"/>
       <c r="Q53" s="4"/>
     </row>
-    <row r="54" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4"/>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3930,7 +3978,7 @@
       <c r="P54" s="4"/>
       <c r="Q54" s="4"/>
     </row>
-    <row r="55" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3949,7 +3997,7 @@
       <c r="P55" s="4"/>
       <c r="Q55" s="4"/>
     </row>
-    <row r="56" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -3968,7 +4016,7 @@
       <c r="P56" s="4"/>
       <c r="Q56" s="4"/>
     </row>
-    <row r="57" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -3987,7 +4035,7 @@
       <c r="P57" s="4"/>
       <c r="Q57" s="4"/>
     </row>
-    <row r="58" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -4006,7 +4054,7 @@
       <c r="P58" s="4"/>
       <c r="Q58" s="4"/>
     </row>
-    <row r="59" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -4025,7 +4073,7 @@
       <c r="P59" s="4"/>
       <c r="Q59" s="4"/>
     </row>
-    <row r="60" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -4044,7 +4092,7 @@
       <c r="P60" s="4"/>
       <c r="Q60" s="4"/>
     </row>
-    <row r="61" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
@@ -4063,7 +4111,7 @@
       <c r="P61" s="4"/>
       <c r="Q61" s="4"/>
     </row>
-    <row r="62" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -4082,7 +4130,7 @@
       <c r="P62" s="4"/>
       <c r="Q62" s="4"/>
     </row>
-    <row r="63" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -4101,7 +4149,7 @@
       <c r="P63" s="4"/>
       <c r="Q63" s="4"/>
     </row>
-    <row r="64" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -4120,7 +4168,7 @@
       <c r="P64" s="4"/>
       <c r="Q64" s="4"/>
     </row>
-    <row r="65" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
@@ -4139,7 +4187,7 @@
       <c r="P65" s="4"/>
       <c r="Q65" s="4"/>
     </row>
-    <row r="66" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -4158,7 +4206,7 @@
       <c r="P66" s="4"/>
       <c r="Q66" s="4"/>
     </row>
-    <row r="67" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -4177,7 +4225,7 @@
       <c r="P67" s="4"/>
       <c r="Q67" s="4"/>
     </row>
-    <row r="68" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" s="4"/>
       <c r="C68" s="4"/>
@@ -4196,7 +4244,7 @@
       <c r="P68" s="4"/>
       <c r="Q68" s="4"/>
     </row>
-    <row r="69" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" s="4"/>
       <c r="C69" s="4"/>
@@ -4215,7 +4263,7 @@
       <c r="P69" s="4"/>
       <c r="Q69" s="4"/>
     </row>
-    <row r="70" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4"/>
       <c r="B70" s="4"/>
       <c r="C70" s="4"/>
@@ -4234,7 +4282,7 @@
       <c r="P70" s="4"/>
       <c r="Q70" s="4"/>
     </row>
-    <row r="71" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4"/>
       <c r="B71" s="4"/>
       <c r="C71" s="4"/>
@@ -4253,7 +4301,7 @@
       <c r="P71" s="4"/>
       <c r="Q71" s="4"/>
     </row>
-    <row r="72" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" s="4"/>
       <c r="C72" s="4"/>
@@ -4272,7 +4320,7 @@
       <c r="P72" s="4"/>
       <c r="Q72" s="4"/>
     </row>
-    <row r="73" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" s="4"/>
       <c r="C73" s="4"/>
@@ -4291,7 +4339,7 @@
       <c r="P73" s="4"/>
       <c r="Q73" s="4"/>
     </row>
-    <row r="74" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" s="4"/>
       <c r="C74" s="4"/>
@@ -4310,7 +4358,7 @@
       <c r="P74" s="4"/>
       <c r="Q74" s="4"/>
     </row>
-    <row r="75" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" s="4"/>
       <c r="C75" s="4"/>
@@ -4329,7 +4377,7 @@
       <c r="P75" s="4"/>
       <c r="Q75" s="4"/>
     </row>
-    <row r="76" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
       <c r="B76" s="4"/>
       <c r="C76" s="4"/>
@@ -4348,7 +4396,7 @@
       <c r="P76" s="4"/>
       <c r="Q76" s="4"/>
     </row>
-    <row r="77" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" s="4"/>
       <c r="C77" s="4"/>
@@ -4367,7 +4415,7 @@
       <c r="P77" s="4"/>
       <c r="Q77" s="4"/>
     </row>
-    <row r="78" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" s="4"/>
       <c r="C78" s="4"/>
@@ -4386,7 +4434,7 @@
       <c r="P78" s="4"/>
       <c r="Q78" s="4"/>
     </row>
-    <row r="79" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" s="4"/>
       <c r="C79" s="4"/>
@@ -4405,7 +4453,7 @@
       <c r="P79" s="4"/>
       <c r="Q79" s="4"/>
     </row>
-    <row r="80" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
       <c r="B80" s="4"/>
       <c r="C80" s="4"/>
@@ -4424,7 +4472,7 @@
       <c r="P80" s="4"/>
       <c r="Q80" s="4"/>
     </row>
-    <row r="81" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4"/>
       <c r="B81" s="4"/>
       <c r="C81" s="4"/>
@@ -4443,7 +4491,7 @@
       <c r="P81" s="4"/>
       <c r="Q81" s="4"/>
     </row>
-    <row r="82" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" s="4"/>
       <c r="C82" s="4"/>
@@ -4462,7 +4510,7 @@
       <c r="P82" s="4"/>
       <c r="Q82" s="4"/>
     </row>
-    <row r="83" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4"/>
       <c r="B83" s="4"/>
       <c r="C83" s="4"/>
@@ -4481,7 +4529,7 @@
       <c r="P83" s="4"/>
       <c r="Q83" s="4"/>
     </row>
-    <row r="84" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4"/>
       <c r="B84" s="4"/>
       <c r="C84" s="4"/>
@@ -4500,7 +4548,7 @@
       <c r="P84" s="4"/>
       <c r="Q84" s="4"/>
     </row>
-    <row r="85" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4"/>
       <c r="B85" s="4"/>
       <c r="C85" s="4"/>
@@ -4519,7 +4567,7 @@
       <c r="P85" s="4"/>
       <c r="Q85" s="4"/>
     </row>
-    <row r="86" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4"/>
       <c r="B86" s="4"/>
       <c r="C86" s="4"/>
@@ -4538,7 +4586,7 @@
       <c r="P86" s="4"/>
       <c r="Q86" s="4"/>
     </row>
-    <row r="87" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4"/>
       <c r="B87" s="4"/>
       <c r="C87" s="4"/>
@@ -4557,7 +4605,7 @@
       <c r="P87" s="4"/>
       <c r="Q87" s="4"/>
     </row>
-    <row r="88" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4"/>
       <c r="B88" s="4"/>
       <c r="C88" s="4"/>
@@ -4576,7 +4624,7 @@
       <c r="P88" s="4"/>
       <c r="Q88" s="4"/>
     </row>
-    <row r="89" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4"/>
       <c r="B89" s="4"/>
       <c r="C89" s="4"/>
@@ -4595,7 +4643,7 @@
       <c r="P89" s="4"/>
       <c r="Q89" s="4"/>
     </row>
-    <row r="90" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4"/>
       <c r="B90" s="4"/>
       <c r="C90" s="4"/>
@@ -4614,7 +4662,7 @@
       <c r="P90" s="4"/>
       <c r="Q90" s="4"/>
     </row>
-    <row r="91" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4"/>
       <c r="B91" s="4"/>
       <c r="C91" s="4"/>
@@ -4633,7 +4681,7 @@
       <c r="P91" s="4"/>
       <c r="Q91" s="4"/>
     </row>
-    <row r="92" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4"/>
       <c r="B92" s="4"/>
       <c r="C92" s="4"/>
@@ -4652,7 +4700,7 @@
       <c r="P92" s="4"/>
       <c r="Q92" s="4"/>
     </row>
-    <row r="93" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4"/>
       <c r="B93" s="4"/>
       <c r="C93" s="4"/>
@@ -4671,7 +4719,7 @@
       <c r="P93" s="4"/>
       <c r="Q93" s="4"/>
     </row>
-    <row r="94" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4"/>
       <c r="B94" s="4"/>
       <c r="C94" s="4"/>
@@ -4690,7 +4738,7 @@
       <c r="P94" s="4"/>
       <c r="Q94" s="4"/>
     </row>
-    <row r="95" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4"/>
       <c r="B95" s="4"/>
       <c r="C95" s="4"/>
@@ -4709,7 +4757,7 @@
       <c r="P95" s="4"/>
       <c r="Q95" s="4"/>
     </row>
-    <row r="96" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="4"/>
       <c r="B96" s="4"/>
       <c r="C96" s="4"/>
@@ -4728,7 +4776,7 @@
       <c r="P96" s="4"/>
       <c r="Q96" s="4"/>
     </row>
-    <row r="97" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="4"/>
       <c r="B97" s="4"/>
       <c r="C97" s="4"/>
@@ -4747,7 +4795,7 @@
       <c r="P97" s="4"/>
       <c r="Q97" s="4"/>
     </row>
-    <row r="98" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4"/>
       <c r="B98" s="4"/>
       <c r="C98" s="4"/>
@@ -4766,7 +4814,7 @@
       <c r="P98" s="4"/>
       <c r="Q98" s="4"/>
     </row>
-    <row r="99" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="4"/>
       <c r="B99" s="4"/>
       <c r="C99" s="4"/>
@@ -4785,7 +4833,7 @@
       <c r="P99" s="4"/>
       <c r="Q99" s="4"/>
     </row>
-    <row r="100" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4"/>
       <c r="B100" s="4"/>
       <c r="C100" s="4"/>
@@ -4804,7 +4852,7 @@
       <c r="P100" s="4"/>
       <c r="Q100" s="4"/>
     </row>
-    <row r="101" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="4"/>
       <c r="B101" s="4"/>
       <c r="C101" s="4"/>
@@ -4823,7 +4871,7 @@
       <c r="P101" s="4"/>
       <c r="Q101" s="4"/>
     </row>
-    <row r="102" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="4"/>
       <c r="B102" s="4"/>
       <c r="C102" s="4"/>
@@ -4842,7 +4890,7 @@
       <c r="P102" s="4"/>
       <c r="Q102" s="4"/>
     </row>
-    <row r="103" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="4"/>
       <c r="B103" s="4"/>
       <c r="C103" s="4"/>
@@ -4861,7 +4909,7 @@
       <c r="P103" s="4"/>
       <c r="Q103" s="4"/>
     </row>
-    <row r="104" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="4"/>
       <c r="B104" s="4"/>
       <c r="C104" s="4"/>
@@ -4880,7 +4928,7 @@
       <c r="P104" s="4"/>
       <c r="Q104" s="4"/>
     </row>
-    <row r="105" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="4"/>
       <c r="B105" s="4"/>
       <c r="C105" s="4"/>
@@ -4899,7 +4947,7 @@
       <c r="P105" s="4"/>
       <c r="Q105" s="4"/>
     </row>
-    <row r="106" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="4"/>
       <c r="B106" s="4"/>
       <c r="C106" s="4"/>
@@ -4918,7 +4966,7 @@
       <c r="P106" s="4"/>
       <c r="Q106" s="4"/>
     </row>
-    <row r="107" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="4"/>
       <c r="B107" s="4"/>
       <c r="C107" s="4"/>
@@ -4937,7 +4985,7 @@
       <c r="P107" s="4"/>
       <c r="Q107" s="4"/>
     </row>
-    <row r="108" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="4"/>
       <c r="B108" s="4"/>
       <c r="C108" s="4"/>
@@ -4956,7 +5004,7 @@
       <c r="P108" s="4"/>
       <c r="Q108" s="4"/>
     </row>
-    <row r="109" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="4"/>
       <c r="B109" s="4"/>
       <c r="C109" s="4"/>
@@ -4975,7 +5023,7 @@
       <c r="P109" s="4"/>
       <c r="Q109" s="4"/>
     </row>
-    <row r="110" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="4"/>
       <c r="B110" s="4"/>
       <c r="C110" s="4"/>
@@ -4994,7 +5042,7 @@
       <c r="P110" s="4"/>
       <c r="Q110" s="4"/>
     </row>
-    <row r="111" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="4"/>
       <c r="B111" s="4"/>
       <c r="C111" s="4"/>
@@ -5013,7 +5061,7 @@
       <c r="P111" s="4"/>
       <c r="Q111" s="4"/>
     </row>
-    <row r="112" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="4"/>
       <c r="B112" s="4"/>
       <c r="C112" s="4"/>
@@ -5032,7 +5080,7 @@
       <c r="P112" s="4"/>
       <c r="Q112" s="4"/>
     </row>
-    <row r="113" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="4"/>
       <c r="B113" s="4"/>
       <c r="C113" s="4"/>
@@ -5051,7 +5099,7 @@
       <c r="P113" s="4"/>
       <c r="Q113" s="4"/>
     </row>
-    <row r="114" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="4"/>
       <c r="B114" s="4"/>
       <c r="C114" s="4"/>
@@ -5070,7 +5118,7 @@
       <c r="P114" s="4"/>
       <c r="Q114" s="4"/>
     </row>
-    <row r="115" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="4"/>
       <c r="B115" s="4"/>
       <c r="C115" s="4"/>
@@ -5089,7 +5137,7 @@
       <c r="P115" s="4"/>
       <c r="Q115" s="4"/>
     </row>
-    <row r="116" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="4"/>
       <c r="B116" s="4"/>
       <c r="C116" s="4"/>
@@ -5108,7 +5156,7 @@
       <c r="P116" s="4"/>
       <c r="Q116" s="4"/>
     </row>
-    <row r="117" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="4"/>
       <c r="B117" s="4"/>
       <c r="C117" s="4"/>
@@ -5127,7 +5175,7 @@
       <c r="P117" s="4"/>
       <c r="Q117" s="4"/>
     </row>
-    <row r="118" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="4"/>
       <c r="B118" s="4"/>
       <c r="C118" s="4"/>
@@ -5146,7 +5194,7 @@
       <c r="P118" s="4"/>
       <c r="Q118" s="4"/>
     </row>
-    <row r="119" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="4"/>
       <c r="B119" s="4"/>
       <c r="C119" s="4"/>
@@ -5165,7 +5213,7 @@
       <c r="P119" s="4"/>
       <c r="Q119" s="4"/>
     </row>
-    <row r="120" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="4"/>
       <c r="B120" s="4"/>
       <c r="C120" s="4"/>
@@ -5184,7 +5232,7 @@
       <c r="P120" s="4"/>
       <c r="Q120" s="4"/>
     </row>
-    <row r="121" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="4"/>
       <c r="B121" s="4"/>
       <c r="C121" s="4"/>
@@ -5203,7 +5251,7 @@
       <c r="P121" s="4"/>
       <c r="Q121" s="4"/>
     </row>
-    <row r="122" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="4"/>
       <c r="B122" s="4"/>
       <c r="C122" s="4"/>
@@ -5222,7 +5270,7 @@
       <c r="P122" s="4"/>
       <c r="Q122" s="4"/>
     </row>
-    <row r="123" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="4"/>
       <c r="B123" s="4"/>
       <c r="C123" s="4"/>
@@ -5241,7 +5289,7 @@
       <c r="P123" s="4"/>
       <c r="Q123" s="4"/>
     </row>
-    <row r="124" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="4"/>
       <c r="B124" s="4"/>
       <c r="C124" s="4"/>
@@ -5260,7 +5308,7 @@
       <c r="P124" s="4"/>
       <c r="Q124" s="4"/>
     </row>
-    <row r="125" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="4"/>
       <c r="B125" s="4"/>
       <c r="C125" s="4"/>
@@ -5279,7 +5327,7 @@
       <c r="P125" s="4"/>
       <c r="Q125" s="4"/>
     </row>
-    <row r="126" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="4"/>
       <c r="B126" s="4"/>
       <c r="C126" s="4"/>
@@ -5298,7 +5346,7 @@
       <c r="P126" s="4"/>
       <c r="Q126" s="4"/>
     </row>
-    <row r="127" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="4"/>
       <c r="B127" s="4"/>
       <c r="C127" s="4"/>
@@ -5317,7 +5365,7 @@
       <c r="P127" s="4"/>
       <c r="Q127" s="4"/>
     </row>
-    <row r="128" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="4"/>
       <c r="B128" s="4"/>
       <c r="C128" s="4"/>
@@ -5336,7 +5384,7 @@
       <c r="P128" s="4"/>
       <c r="Q128" s="4"/>
     </row>
-    <row r="129" spans="1:17" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:17" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="4"/>
       <c r="B129" s="4"/>
       <c r="C129" s="4"/>

</xml_diff>